<commit_message>
K45+500: correct design flood level to 33.89 m
The K45+500 case carried 34.04 m over from the original model input;
the design flood level of this section is 33.89 m.  Crest freeboard is
36.30 - 33.89 = 2.41 m, still above the 2.0 m river requirement, so B1
and all evaluation results are unchanged (C, 22.8; 24.3 with the
stability recompute).

- case indicator table, K45+500 trace ledger, chapter-5 script comment
- levee_eval_api 1.3.2: demo workbook, Excel tests, docs/05 demo table
- data-collection checklist
The 875 synthetic benchmark keeps its fixed 34.04 m setting.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HPr98chDrorJ6AwDwTysfM
</commit_message>
<xml_diff>
--- a/delivery/planning/safety_eval_data_checklist_20261025.xlsx
+++ b/delivery/planning/safety_eval_data_checklist_20261025.xlsx
@@ -574,7 +574,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>K45+500 有（设计洪水位 34.04 m；符合 2 级堤防防洪标准）</t>
+          <t>K45+500 有（设计洪水位 33.89 m；符合 2 级堤防防洪标准）</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>34.04</t>
+          <t>33.89</t>
         </is>
       </c>
     </row>

</xml_diff>